<commit_message>
Execute Step 12: Cluster analysis complete — identified 4 user employability profiles with demographic and behavioral characteristics
</commit_message>
<xml_diff>
--- a/data/ia_comp.xlsx
+++ b/data/ia_comp.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10821"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F59C2BB6-B0B5-44DD-8111-DA238AABEBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C66F59-7FA5-C842-A9D6-5622AE27D2A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Panelists" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4254" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4255" uniqueCount="56">
   <si>
     <t>SEXO</t>
   </si>
@@ -601,9 +601,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O504"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>55</v>
       </c>
@@ -650,7 +650,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -679,7 +679,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -708,7 +708,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -737,7 +737,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -766,7 +766,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -795,7 +795,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -827,7 +827,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -859,7 +859,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -888,7 +888,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -917,7 +917,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -952,7 +952,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -981,7 +981,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1010,7 +1010,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1039,7 +1039,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1068,7 +1068,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1155,7 +1155,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1277,7 +1277,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1344,7 +1344,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1373,7 +1373,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1489,7 +1489,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1582,7 +1582,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1611,7 +1611,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1669,7 +1669,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1904,7 +1904,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1936,7 +1936,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2090,7 +2090,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2250,7 +2250,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2279,7 +2279,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2308,7 +2308,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2369,7 +2369,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2398,7 +2398,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2517,7 +2517,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2575,7 +2575,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2613,7 +2613,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2671,7 +2671,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2877,7 +2877,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2906,7 +2906,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2935,7 +2935,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2964,7 +2964,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A80">
         <v>79</v>
       </c>
@@ -3025,7 +3025,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A81">
         <v>80</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A82">
         <v>81</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A83">
         <v>82</v>
       </c>
@@ -3121,7 +3121,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A84">
         <v>83</v>
       </c>
@@ -3150,7 +3150,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A85">
         <v>84</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A86">
         <v>85</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A87">
         <v>86</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A88">
         <v>87</v>
       </c>
@@ -3266,7 +3266,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A89">
         <v>88</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A90">
         <v>89</v>
       </c>
@@ -3324,7 +3324,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A91">
         <v>90</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A92">
         <v>91</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A93">
         <v>92</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A94">
         <v>93</v>
       </c>
@@ -3440,7 +3440,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3469,7 +3469,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3527,7 +3527,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3556,7 +3556,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3620,7 +3620,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3765,7 +3765,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3896,7 +3896,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3925,7 +3925,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3954,7 +3954,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A112">
         <v>111</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A113">
         <v>112</v>
       </c>
@@ -4015,7 +4015,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A114">
         <v>113</v>
       </c>
@@ -4044,7 +4044,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A115">
         <v>114</v>
       </c>
@@ -4073,7 +4073,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A116">
         <v>115</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A117">
         <v>116</v>
       </c>
@@ -4140,7 +4140,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A118">
         <v>117</v>
       </c>
@@ -4175,7 +4175,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A119">
         <v>118</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A120">
         <v>119</v>
       </c>
@@ -4239,7 +4239,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A121">
         <v>120</v>
       </c>
@@ -4268,7 +4268,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A122">
         <v>121</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A123">
         <v>122</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A124">
         <v>123</v>
       </c>
@@ -4358,7 +4358,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A125">
         <v>124</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A126">
         <v>125</v>
       </c>
@@ -4419,7 +4419,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A127">
         <v>126</v>
       </c>
@@ -4448,7 +4448,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A128">
         <v>127</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A129">
         <v>128</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A130">
         <v>129</v>
       </c>
@@ -4541,7 +4541,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A131">
         <v>130</v>
       </c>
@@ -4570,7 +4570,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A132">
         <v>131</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A133">
         <v>132</v>
       </c>
@@ -4628,7 +4628,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A134">
         <v>133</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A135">
         <v>134</v>
       </c>
@@ -4686,7 +4686,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A136">
         <v>135</v>
       </c>
@@ -4702,6 +4702,9 @@
       <c r="E136" t="s">
         <v>34</v>
       </c>
+      <c r="F136" t="s">
+        <v>39</v>
+      </c>
       <c r="G136" t="s">
         <v>49</v>
       </c>
@@ -4712,7 +4715,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A137">
         <v>136</v>
       </c>
@@ -4741,7 +4744,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A138">
         <v>137</v>
       </c>
@@ -4773,7 +4776,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A139">
         <v>138</v>
       </c>
@@ -4802,7 +4805,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A140">
         <v>139</v>
       </c>
@@ -4834,7 +4837,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A141">
         <v>140</v>
       </c>
@@ -4872,7 +4875,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A142">
         <v>141</v>
       </c>
@@ -4901,7 +4904,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A143">
         <v>142</v>
       </c>
@@ -4930,7 +4933,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A144">
         <v>143</v>
       </c>
@@ -4959,7 +4962,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A145">
         <v>144</v>
       </c>
@@ -4988,7 +4991,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A146">
         <v>145</v>
       </c>
@@ -5017,7 +5020,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A147">
         <v>146</v>
       </c>
@@ -5046,7 +5049,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A148">
         <v>147</v>
       </c>
@@ -5075,7 +5078,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A149">
         <v>148</v>
       </c>
@@ -5113,7 +5116,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A150">
         <v>149</v>
       </c>
@@ -5142,7 +5145,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A151">
         <v>150</v>
       </c>
@@ -5171,7 +5174,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A152">
         <v>151</v>
       </c>
@@ -5200,7 +5203,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A153">
         <v>152</v>
       </c>
@@ -5229,7 +5232,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A154">
         <v>153</v>
       </c>
@@ -5258,7 +5261,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A155">
         <v>154</v>
       </c>
@@ -5287,7 +5290,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A156">
         <v>155</v>
       </c>
@@ -5316,7 +5319,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A157">
         <v>156</v>
       </c>
@@ -5345,7 +5348,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A158">
         <v>157</v>
       </c>
@@ -5374,7 +5377,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A159">
         <v>158</v>
       </c>
@@ -5403,7 +5406,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A160">
         <v>159</v>
       </c>
@@ -5432,7 +5435,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A161">
         <v>160</v>
       </c>
@@ -5464,7 +5467,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A162">
         <v>161</v>
       </c>
@@ -5493,7 +5496,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A163">
         <v>162</v>
       </c>
@@ -5522,7 +5525,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A164">
         <v>163</v>
       </c>
@@ -5551,7 +5554,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A165">
         <v>164</v>
       </c>
@@ -5580,7 +5583,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A166">
         <v>165</v>
       </c>
@@ -5612,7 +5615,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A167">
         <v>166</v>
       </c>
@@ -5644,7 +5647,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A168">
         <v>167</v>
       </c>
@@ -5676,7 +5679,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A169">
         <v>168</v>
       </c>
@@ -5705,7 +5708,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A170">
         <v>169</v>
       </c>
@@ -5734,7 +5737,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A171">
         <v>170</v>
       </c>
@@ -5763,7 +5766,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A172">
         <v>171</v>
       </c>
@@ -5792,7 +5795,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A173">
         <v>172</v>
       </c>
@@ -5821,7 +5824,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A174">
         <v>173</v>
       </c>
@@ -5850,7 +5853,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A175">
         <v>174</v>
       </c>
@@ -5879,7 +5882,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A176">
         <v>175</v>
       </c>
@@ -5908,7 +5911,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A177">
         <v>176</v>
       </c>
@@ -5937,7 +5940,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A178">
         <v>177</v>
       </c>
@@ -5966,7 +5969,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A179">
         <v>178</v>
       </c>
@@ -5995,7 +5998,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A180">
         <v>179</v>
       </c>
@@ -6024,7 +6027,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A181">
         <v>180</v>
       </c>
@@ -6053,7 +6056,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A182">
         <v>181</v>
       </c>
@@ -6082,7 +6085,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A183">
         <v>182</v>
       </c>
@@ -6111,7 +6114,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A184">
         <v>183</v>
       </c>
@@ -6140,7 +6143,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A185">
         <v>184</v>
       </c>
@@ -6169,7 +6172,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A186">
         <v>185</v>
       </c>
@@ -6198,7 +6201,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A187">
         <v>186</v>
       </c>
@@ -6233,7 +6236,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A188">
         <v>187</v>
       </c>
@@ -6262,7 +6265,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A189">
         <v>188</v>
       </c>
@@ -6291,7 +6294,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A190">
         <v>189</v>
       </c>
@@ -6320,7 +6323,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A191">
         <v>190</v>
       </c>
@@ -6349,7 +6352,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A192">
         <v>191</v>
       </c>
@@ -6378,7 +6381,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A193">
         <v>192</v>
       </c>
@@ -6407,7 +6410,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A194">
         <v>193</v>
       </c>
@@ -6436,7 +6439,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A195">
         <v>194</v>
       </c>
@@ -6471,7 +6474,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A196">
         <v>195</v>
       </c>
@@ -6500,7 +6503,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A197">
         <v>196</v>
       </c>
@@ -6529,7 +6532,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A198">
         <v>197</v>
       </c>
@@ -6558,7 +6561,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A199">
         <v>198</v>
       </c>
@@ -6587,7 +6590,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A200">
         <v>199</v>
       </c>
@@ -6619,7 +6622,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A201">
         <v>200</v>
       </c>
@@ -6648,7 +6651,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A202">
         <v>201</v>
       </c>
@@ -6677,7 +6680,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A203">
         <v>202</v>
       </c>
@@ -6709,7 +6712,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A204">
         <v>203</v>
       </c>
@@ -6738,7 +6741,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A205">
         <v>204</v>
       </c>
@@ -6773,7 +6776,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A206">
         <v>205</v>
       </c>
@@ -6811,7 +6814,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A207">
         <v>206</v>
       </c>
@@ -6840,7 +6843,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A208">
         <v>207</v>
       </c>
@@ -6869,7 +6872,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A209">
         <v>208</v>
       </c>
@@ -6898,7 +6901,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A210">
         <v>209</v>
       </c>
@@ -6927,7 +6930,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A211">
         <v>210</v>
       </c>
@@ -6959,7 +6962,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A212">
         <v>211</v>
       </c>
@@ -6988,7 +6991,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A213">
         <v>212</v>
       </c>
@@ -7017,7 +7020,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A214">
         <v>213</v>
       </c>
@@ -7046,7 +7049,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A215">
         <v>214</v>
       </c>
@@ -7075,7 +7078,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A216">
         <v>215</v>
       </c>
@@ -7104,7 +7107,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A217">
         <v>216</v>
       </c>
@@ -7133,7 +7136,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A218">
         <v>217</v>
       </c>
@@ -7162,7 +7165,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A219">
         <v>218</v>
       </c>
@@ -7194,7 +7197,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A220">
         <v>219</v>
       </c>
@@ -7226,7 +7229,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A221">
         <v>220</v>
       </c>
@@ -7255,7 +7258,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A222">
         <v>221</v>
       </c>
@@ -7284,7 +7287,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A223">
         <v>222</v>
       </c>
@@ -7322,7 +7325,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A224">
         <v>223</v>
       </c>
@@ -7354,7 +7357,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="225" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A225">
         <v>224</v>
       </c>
@@ -7383,7 +7386,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="226" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A226">
         <v>225</v>
       </c>
@@ -7415,7 +7418,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="227" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A227">
         <v>226</v>
       </c>
@@ -7444,7 +7447,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="228" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A228">
         <v>227</v>
       </c>
@@ -7473,7 +7476,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="229" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A229">
         <v>228</v>
       </c>
@@ -7508,7 +7511,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="230" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A230">
         <v>229</v>
       </c>
@@ -7537,7 +7540,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="231" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A231">
         <v>230</v>
       </c>
@@ -7566,7 +7569,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="232" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A232">
         <v>231</v>
       </c>
@@ -7604,7 +7607,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="233" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A233">
         <v>232</v>
       </c>
@@ -7636,7 +7639,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="234" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A234">
         <v>233</v>
       </c>
@@ -7671,7 +7674,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="235" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A235">
         <v>234</v>
       </c>
@@ -7703,7 +7706,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="236" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A236">
         <v>235</v>
       </c>
@@ -7732,7 +7735,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="237" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A237">
         <v>236</v>
       </c>
@@ -7761,7 +7764,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="238" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A238">
         <v>237</v>
       </c>
@@ -7790,7 +7793,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="239" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A239">
         <v>238</v>
       </c>
@@ -7822,7 +7825,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="240" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A240">
         <v>239</v>
       </c>
@@ -7851,7 +7854,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="241" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A241">
         <v>240</v>
       </c>
@@ -7880,7 +7883,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="242" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A242">
         <v>241</v>
       </c>
@@ -7909,7 +7912,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="243" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A243">
         <v>242</v>
       </c>
@@ -7941,7 +7944,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="244" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A244">
         <v>243</v>
       </c>
@@ -7979,7 +7982,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="245" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A245">
         <v>244</v>
       </c>
@@ -8008,7 +8011,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="246" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A246">
         <v>245</v>
       </c>
@@ -8046,7 +8049,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="247" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A247">
         <v>246</v>
       </c>
@@ -8081,7 +8084,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="248" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A248">
         <v>247</v>
       </c>
@@ -8110,7 +8113,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="249" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A249">
         <v>248</v>
       </c>
@@ -8145,7 +8148,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="250" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A250">
         <v>249</v>
       </c>
@@ -8177,7 +8180,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="251" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A251">
         <v>250</v>
       </c>
@@ -8206,7 +8209,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="252" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A252">
         <v>251</v>
       </c>
@@ -8235,7 +8238,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="253" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A253">
         <v>252</v>
       </c>
@@ -8264,7 +8267,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="254" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A254">
         <v>253</v>
       </c>
@@ -8293,7 +8296,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="255" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A255">
         <v>254</v>
       </c>
@@ -8328,7 +8331,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="256" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A256">
         <v>255</v>
       </c>
@@ -8357,7 +8360,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="257" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A257">
         <v>256</v>
       </c>
@@ -8395,7 +8398,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="258" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A258">
         <v>257</v>
       </c>
@@ -8430,7 +8433,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="259" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A259">
         <v>258</v>
       </c>
@@ -8459,7 +8462,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="260" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A260">
         <v>259</v>
       </c>
@@ -8488,7 +8491,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="261" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A261">
         <v>260</v>
       </c>
@@ -8517,7 +8520,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="262" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A262">
         <v>261</v>
       </c>
@@ -8546,7 +8549,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="263" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A263">
         <v>262</v>
       </c>
@@ -8581,7 +8584,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="264" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A264">
         <v>263</v>
       </c>
@@ -8616,7 +8619,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="265" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A265">
         <v>264</v>
       </c>
@@ -8645,7 +8648,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="266" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A266">
         <v>265</v>
       </c>
@@ -8674,7 +8677,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="267" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A267">
         <v>266</v>
       </c>
@@ -8703,7 +8706,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="268" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A268">
         <v>267</v>
       </c>
@@ -8741,7 +8744,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="269" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A269">
         <v>268</v>
       </c>
@@ -8770,7 +8773,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="270" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A270">
         <v>269</v>
       </c>
@@ -8799,7 +8802,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="271" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A271">
         <v>270</v>
       </c>
@@ -8828,7 +8831,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="272" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A272">
         <v>271</v>
       </c>
@@ -8857,7 +8860,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="273" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A273">
         <v>272</v>
       </c>
@@ -8886,7 +8889,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="274" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A274">
         <v>273</v>
       </c>
@@ -8915,7 +8918,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="275" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A275">
         <v>274</v>
       </c>
@@ -8944,7 +8947,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="276" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A276">
         <v>275</v>
       </c>
@@ -8973,7 +8976,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="277" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A277">
         <v>276</v>
       </c>
@@ -9002,7 +9005,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="278" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A278">
         <v>277</v>
       </c>
@@ -9031,7 +9034,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="279" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A279">
         <v>278</v>
       </c>
@@ -9060,7 +9063,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="280" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A280">
         <v>279</v>
       </c>
@@ -9089,7 +9092,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="281" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A281">
         <v>280</v>
       </c>
@@ -9118,7 +9121,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="282" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A282">
         <v>281</v>
       </c>
@@ -9147,7 +9150,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="283" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A283">
         <v>282</v>
       </c>
@@ -9176,7 +9179,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="284" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A284">
         <v>283</v>
       </c>
@@ -9208,7 +9211,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="285" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A285">
         <v>284</v>
       </c>
@@ -9237,7 +9240,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="286" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A286">
         <v>285</v>
       </c>
@@ -9266,7 +9269,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="287" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A287">
         <v>286</v>
       </c>
@@ -9298,7 +9301,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="288" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A288">
         <v>287</v>
       </c>
@@ -9327,7 +9330,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="289" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A289">
         <v>288</v>
       </c>
@@ -9356,7 +9359,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="290" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A290">
         <v>289</v>
       </c>
@@ -9385,7 +9388,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="291" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A291">
         <v>290</v>
       </c>
@@ -9414,7 +9417,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="292" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A292">
         <v>291</v>
       </c>
@@ -9446,7 +9449,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="293" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A293">
         <v>292</v>
       </c>
@@ -9481,7 +9484,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="294" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A294">
         <v>293</v>
       </c>
@@ -9510,7 +9513,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="295" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A295">
         <v>294</v>
       </c>
@@ -9545,7 +9548,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="296" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A296">
         <v>295</v>
       </c>
@@ -9574,7 +9577,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="297" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A297">
         <v>296</v>
       </c>
@@ -9603,7 +9606,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="298" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A298">
         <v>297</v>
       </c>
@@ -9632,7 +9635,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="299" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A299">
         <v>298</v>
       </c>
@@ -9661,7 +9664,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="300" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A300">
         <v>299</v>
       </c>
@@ -9690,7 +9693,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="301" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A301">
         <v>300</v>
       </c>
@@ -9719,7 +9722,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="302" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A302">
         <v>301</v>
       </c>
@@ -9748,7 +9751,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="303" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A303">
         <v>302</v>
       </c>
@@ -9777,7 +9780,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="304" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A304">
         <v>303</v>
       </c>
@@ -9812,7 +9815,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A305">
         <v>304</v>
       </c>
@@ -9841,7 +9844,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A306">
         <v>305</v>
       </c>
@@ -9870,7 +9873,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A307">
         <v>306</v>
       </c>
@@ -9905,7 +9908,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A308">
         <v>307</v>
       </c>
@@ -9934,7 +9937,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A309">
         <v>308</v>
       </c>
@@ -9963,7 +9966,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="310" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A310">
         <v>309</v>
       </c>
@@ -9995,7 +9998,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="311" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A311">
         <v>310</v>
       </c>
@@ -10024,7 +10027,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="312" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A312">
         <v>311</v>
       </c>
@@ -10053,7 +10056,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="313" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A313">
         <v>312</v>
       </c>
@@ -10082,7 +10085,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="314" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A314">
         <v>313</v>
       </c>
@@ -10111,7 +10114,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="315" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A315">
         <v>314</v>
       </c>
@@ -10140,7 +10143,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="316" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A316">
         <v>315</v>
       </c>
@@ -10169,7 +10172,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="317" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A317">
         <v>316</v>
       </c>
@@ -10198,7 +10201,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="318" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A318">
         <v>317</v>
       </c>
@@ -10227,7 +10230,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="319" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A319">
         <v>318</v>
       </c>
@@ -10256,7 +10259,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="320" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A320">
         <v>319</v>
       </c>
@@ -10288,7 +10291,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="321" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A321">
         <v>320</v>
       </c>
@@ -10317,7 +10320,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="322" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A322">
         <v>321</v>
       </c>
@@ -10346,7 +10349,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="323" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A323">
         <v>322</v>
       </c>
@@ -10375,7 +10378,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="324" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A324">
         <v>323</v>
       </c>
@@ -10404,7 +10407,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="325" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A325">
         <v>324</v>
       </c>
@@ -10433,7 +10436,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="326" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A326">
         <v>325</v>
       </c>
@@ -10462,7 +10465,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="327" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A327">
         <v>326</v>
       </c>
@@ -10491,7 +10494,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="328" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A328">
         <v>327</v>
       </c>
@@ -10520,7 +10523,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="329" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A329">
         <v>328</v>
       </c>
@@ -10549,7 +10552,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="330" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A330">
         <v>329</v>
       </c>
@@ -10578,7 +10581,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="331" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A331">
         <v>330</v>
       </c>
@@ -10607,7 +10610,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="332" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A332">
         <v>331</v>
       </c>
@@ -10636,7 +10639,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="333" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A333">
         <v>332</v>
       </c>
@@ -10665,7 +10668,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="334" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A334">
         <v>333</v>
       </c>
@@ -10694,7 +10697,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="335" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A335">
         <v>334</v>
       </c>
@@ -10723,7 +10726,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="336" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A336">
         <v>335</v>
       </c>
@@ -10752,7 +10755,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="337" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A337">
         <v>336</v>
       </c>
@@ -10790,7 +10793,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="338" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A338">
         <v>337</v>
       </c>
@@ -10825,7 +10828,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="339" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A339">
         <v>338</v>
       </c>
@@ -10854,7 +10857,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="340" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A340">
         <v>339</v>
       </c>
@@ -10883,7 +10886,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="341" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A341">
         <v>340</v>
       </c>
@@ -10915,7 +10918,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="342" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A342">
         <v>341</v>
       </c>
@@ -10944,7 +10947,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="343" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A343">
         <v>342</v>
       </c>
@@ -10973,7 +10976,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="344" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A344">
         <v>343</v>
       </c>
@@ -11008,7 +11011,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="345" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A345">
         <v>344</v>
       </c>
@@ -11040,7 +11043,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="346" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A346">
         <v>345</v>
       </c>
@@ -11069,7 +11072,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="347" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A347">
         <v>346</v>
       </c>
@@ -11098,7 +11101,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="348" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A348">
         <v>347</v>
       </c>
@@ -11127,7 +11130,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="349" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A349">
         <v>348</v>
       </c>
@@ -11156,7 +11159,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="350" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A350">
         <v>349</v>
       </c>
@@ -11185,7 +11188,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="351" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A351">
         <v>350</v>
       </c>
@@ -11214,7 +11217,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="352" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A352">
         <v>351</v>
       </c>
@@ -11243,7 +11246,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="353" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A353">
         <v>352</v>
       </c>
@@ -11272,7 +11275,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="354" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="354" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A354">
         <v>353</v>
       </c>
@@ -11301,7 +11304,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="355" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="355" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A355">
         <v>354</v>
       </c>
@@ -11339,7 +11342,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="356" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A356">
         <v>355</v>
       </c>
@@ -11368,7 +11371,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="357" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A357">
         <v>356</v>
       </c>
@@ -11397,7 +11400,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="358" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A358">
         <v>357</v>
       </c>
@@ -11426,7 +11429,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="359" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A359">
         <v>358</v>
       </c>
@@ -11461,7 +11464,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="360" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A360">
         <v>359</v>
       </c>
@@ -11490,7 +11493,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="361" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="361" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A361">
         <v>360</v>
       </c>
@@ -11519,7 +11522,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="362" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="362" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A362">
         <v>361</v>
       </c>
@@ -11551,7 +11554,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="363" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="363" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A363">
         <v>362</v>
       </c>
@@ -11583,7 +11586,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="364" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="364" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A364">
         <v>363</v>
       </c>
@@ -11612,7 +11615,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="365" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A365">
         <v>364</v>
       </c>
@@ -11641,7 +11644,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="366" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A366">
         <v>365</v>
       </c>
@@ -11670,7 +11673,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="367" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A367">
         <v>366</v>
       </c>
@@ -11699,7 +11702,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="368" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A368">
         <v>367</v>
       </c>
@@ -11728,7 +11731,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="369" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A369">
         <v>368</v>
       </c>
@@ -11757,7 +11760,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="370" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A370">
         <v>369</v>
       </c>
@@ -11786,7 +11789,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="371" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="371" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A371">
         <v>370</v>
       </c>
@@ -11815,7 +11818,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="372" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="372" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A372">
         <v>371</v>
       </c>
@@ -11844,7 +11847,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="373" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="373" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A373">
         <v>372</v>
       </c>
@@ -11882,7 +11885,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="374" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A374">
         <v>373</v>
       </c>
@@ -11914,7 +11917,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="375" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A375">
         <v>374</v>
       </c>
@@ -11943,7 +11946,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="376" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A376">
         <v>375</v>
       </c>
@@ -11981,7 +11984,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="377" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A377">
         <v>376</v>
       </c>
@@ -12010,7 +12013,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="378" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A378">
         <v>377</v>
       </c>
@@ -12039,7 +12042,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="379" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="379" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A379">
         <v>378</v>
       </c>
@@ -12068,7 +12071,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="380" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="380" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A380">
         <v>379</v>
       </c>
@@ -12097,7 +12100,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="381" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="381" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A381">
         <v>380</v>
       </c>
@@ -12126,7 +12129,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="382" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="382" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A382">
         <v>381</v>
       </c>
@@ -12164,7 +12167,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="383" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A383">
         <v>382</v>
       </c>
@@ -12193,7 +12196,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="384" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A384">
         <v>383</v>
       </c>
@@ -12222,7 +12225,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="385" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A385">
         <v>384</v>
       </c>
@@ -12251,7 +12254,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="386" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A386">
         <v>385</v>
       </c>
@@ -12280,7 +12283,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="387" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A387">
         <v>386</v>
       </c>
@@ -12309,7 +12312,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="388" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="388" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A388">
         <v>387</v>
       </c>
@@ -12338,7 +12341,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="389" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="389" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A389">
         <v>388</v>
       </c>
@@ -12370,7 +12373,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="390" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="390" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A390">
         <v>389</v>
       </c>
@@ -12399,7 +12402,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="391" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="391" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A391">
         <v>390</v>
       </c>
@@ -12428,7 +12431,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="392" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A392">
         <v>391</v>
       </c>
@@ -12457,7 +12460,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="393" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A393">
         <v>392</v>
       </c>
@@ -12489,7 +12492,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="394" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A394">
         <v>393</v>
       </c>
@@ -12518,7 +12521,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="395" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A395">
         <v>394</v>
       </c>
@@ -12547,7 +12550,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="396" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A396">
         <v>395</v>
       </c>
@@ -12576,7 +12579,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="397" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="397" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A397">
         <v>396</v>
       </c>
@@ -12605,7 +12608,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="398" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="398" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A398">
         <v>397</v>
       </c>
@@ -12634,7 +12637,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="399" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="399" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A399">
         <v>398</v>
       </c>
@@ -12663,7 +12666,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="400" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A400">
         <v>399</v>
       </c>
@@ -12695,7 +12698,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="401" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="401" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A401">
         <v>400</v>
       </c>
@@ -12727,7 +12730,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="402" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="402" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A402">
         <v>401</v>
       </c>
@@ -12756,7 +12759,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="403" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="403" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A403">
         <v>402</v>
       </c>
@@ -12785,7 +12788,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="404" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="404" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A404">
         <v>403</v>
       </c>
@@ -12814,7 +12817,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="405" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="405" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A405">
         <v>404</v>
       </c>
@@ -12843,7 +12846,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="406" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A406">
         <v>405</v>
       </c>
@@ -12872,7 +12875,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="407" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="407" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A407">
         <v>406</v>
       </c>
@@ -12901,7 +12904,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="408" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="408" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A408">
         <v>407</v>
       </c>
@@ -12933,7 +12936,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="409" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="409" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A409">
         <v>408</v>
       </c>
@@ -12968,7 +12971,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="410" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="410" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A410">
         <v>409</v>
       </c>
@@ -13000,7 +13003,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="411" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="411" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A411">
         <v>410</v>
       </c>
@@ -13035,7 +13038,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="412" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="412" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A412">
         <v>411</v>
       </c>
@@ -13064,7 +13067,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="413" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="413" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A413">
         <v>412</v>
       </c>
@@ -13093,7 +13096,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="414" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="414" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A414">
         <v>413</v>
       </c>
@@ -13122,7 +13125,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="415" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="415" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A415">
         <v>414</v>
       </c>
@@ -13151,7 +13154,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="416" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="416" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A416">
         <v>415</v>
       </c>
@@ -13180,7 +13183,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="417" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="417" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A417">
         <v>416</v>
       </c>
@@ -13209,7 +13212,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="418" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="418" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A418">
         <v>417</v>
       </c>
@@ -13238,7 +13241,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="419" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="419" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A419">
         <v>418</v>
       </c>
@@ -13267,7 +13270,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="420" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="420" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A420">
         <v>419</v>
       </c>
@@ -13302,7 +13305,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="421" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="421" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A421">
         <v>420</v>
       </c>
@@ -13334,7 +13337,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="422" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="422" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A422">
         <v>421</v>
       </c>
@@ -13366,7 +13369,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="423" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="423" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A423">
         <v>422</v>
       </c>
@@ -13395,7 +13398,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="424" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="424" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A424">
         <v>423</v>
       </c>
@@ -13430,7 +13433,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="425" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="425" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A425">
         <v>424</v>
       </c>
@@ -13459,7 +13462,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="426" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="426" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A426">
         <v>425</v>
       </c>
@@ -13494,7 +13497,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="427" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="427" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A427">
         <v>426</v>
       </c>
@@ -13526,7 +13529,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="428" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="428" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A428">
         <v>427</v>
       </c>
@@ -13558,7 +13561,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="429" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="429" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A429">
         <v>428</v>
       </c>
@@ -13587,7 +13590,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="430" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="430" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A430">
         <v>429</v>
       </c>
@@ -13616,7 +13619,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="431" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A431">
         <v>430</v>
       </c>
@@ -13654,7 +13657,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="432" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="432" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A432">
         <v>431</v>
       </c>
@@ -13683,7 +13686,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="433" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="433" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A433">
         <v>432</v>
       </c>
@@ -13712,7 +13715,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="434" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="434" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A434">
         <v>433</v>
       </c>
@@ -13741,7 +13744,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="435" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="435" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A435">
         <v>434</v>
       </c>
@@ -13773,7 +13776,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="436" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="436" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A436">
         <v>435</v>
       </c>
@@ -13802,7 +13805,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="437" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="437" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A437">
         <v>436</v>
       </c>
@@ -13831,7 +13834,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="438" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="438" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A438">
         <v>437</v>
       </c>
@@ -13860,7 +13863,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="439" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="439" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A439">
         <v>438</v>
       </c>
@@ -13898,7 +13901,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="440" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="440" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A440">
         <v>439</v>
       </c>
@@ -13927,7 +13930,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="441" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="441" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A441">
         <v>440</v>
       </c>
@@ -13956,7 +13959,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="442" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="442" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A442">
         <v>441</v>
       </c>
@@ -13985,7 +13988,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="443" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="443" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A443">
         <v>442</v>
       </c>
@@ -14014,7 +14017,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="444" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="444" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A444">
         <v>443</v>
       </c>
@@ -14043,7 +14046,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="445" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="445" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A445">
         <v>444</v>
       </c>
@@ -14072,7 +14075,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="446" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="446" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A446">
         <v>445</v>
       </c>
@@ -14101,7 +14104,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="447" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="447" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A447">
         <v>446</v>
       </c>
@@ -14130,7 +14133,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="448" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="448" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A448">
         <v>447</v>
       </c>
@@ -14159,7 +14162,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="449" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="449" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A449">
         <v>448</v>
       </c>
@@ -14191,7 +14194,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="450" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="450" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A450">
         <v>449</v>
       </c>
@@ -14220,7 +14223,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="451" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="451" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A451">
         <v>450</v>
       </c>
@@ -14249,7 +14252,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="452" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="452" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A452">
         <v>451</v>
       </c>
@@ -14278,7 +14281,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="453" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="453" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A453">
         <v>452</v>
       </c>
@@ -14307,7 +14310,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="454" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="454" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A454">
         <v>453</v>
       </c>
@@ -14336,7 +14339,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="455" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="455" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A455">
         <v>454</v>
       </c>
@@ -14365,7 +14368,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="456" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="456" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A456">
         <v>455</v>
       </c>
@@ -14394,7 +14397,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="457" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="457" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A457">
         <v>456</v>
       </c>
@@ -14423,7 +14426,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="458" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="458" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A458">
         <v>457</v>
       </c>
@@ -14458,7 +14461,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="459" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="459" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A459">
         <v>458</v>
       </c>
@@ -14493,7 +14496,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="460" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="460" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A460">
         <v>459</v>
       </c>
@@ -14528,7 +14531,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="461" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="461" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A461">
         <v>460</v>
       </c>
@@ -14566,7 +14569,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="462" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="462" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A462">
         <v>461</v>
       </c>
@@ -14595,7 +14598,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="463" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="463" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A463">
         <v>462</v>
       </c>
@@ -14624,7 +14627,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="464" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="464" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A464">
         <v>463</v>
       </c>
@@ -14653,7 +14656,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="465" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="465" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A465">
         <v>464</v>
       </c>
@@ -14682,7 +14685,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="466" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="466" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A466">
         <v>465</v>
       </c>
@@ -14711,7 +14714,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="467" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="467" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A467">
         <v>466</v>
       </c>
@@ -14743,7 +14746,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="468" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="468" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A468">
         <v>467</v>
       </c>
@@ -14775,7 +14778,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="469" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="469" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A469">
         <v>468</v>
       </c>
@@ -14804,7 +14807,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="470" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="470" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A470">
         <v>469</v>
       </c>
@@ -14833,7 +14836,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="471" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="471" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A471">
         <v>470</v>
       </c>
@@ -14865,7 +14868,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="472" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="472" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A472">
         <v>471</v>
       </c>
@@ -14894,7 +14897,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="473" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="473" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A473">
         <v>472</v>
       </c>
@@ -14923,7 +14926,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="474" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="474" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A474">
         <v>473</v>
       </c>
@@ -14955,7 +14958,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="475" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="475" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A475">
         <v>474</v>
       </c>
@@ -14984,7 +14987,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="476" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="476" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A476">
         <v>475</v>
       </c>
@@ -15016,7 +15019,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="477" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="477" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A477">
         <v>476</v>
       </c>
@@ -15045,7 +15048,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="478" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="478" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A478">
         <v>477</v>
       </c>
@@ -15074,7 +15077,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="479" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="479" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A479">
         <v>478</v>
       </c>
@@ -15103,7 +15106,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="480" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="480" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A480">
         <v>479</v>
       </c>
@@ -15132,7 +15135,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="481" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="481" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A481">
         <v>480</v>
       </c>
@@ -15164,7 +15167,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="482" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="482" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A482">
         <v>481</v>
       </c>
@@ -15193,7 +15196,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="483" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="483" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A483">
         <v>482</v>
       </c>
@@ -15222,7 +15225,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="484" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="484" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A484">
         <v>483</v>
       </c>
@@ -15251,7 +15254,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="485" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="485" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A485">
         <v>484</v>
       </c>
@@ -15286,7 +15289,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="486" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="486" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A486">
         <v>485</v>
       </c>
@@ -15315,7 +15318,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="487" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="487" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A487">
         <v>486</v>
       </c>
@@ -15344,7 +15347,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="488" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="488" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A488">
         <v>487</v>
       </c>
@@ -15382,7 +15385,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="489" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="489" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A489">
         <v>488</v>
       </c>
@@ -15411,7 +15414,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="490" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="490" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A490">
         <v>489</v>
       </c>
@@ -15440,7 +15443,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="491" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="491" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A491">
         <v>490</v>
       </c>
@@ -15469,7 +15472,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="492" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="492" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A492">
         <v>491</v>
       </c>
@@ -15504,7 +15507,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="493" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="493" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A493">
         <v>492</v>
       </c>
@@ -15533,7 +15536,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="494" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="494" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A494">
         <v>493</v>
       </c>
@@ -15562,7 +15565,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="495" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="495" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A495">
         <v>494</v>
       </c>
@@ -15591,7 +15594,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="496" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="496" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A496">
         <v>495</v>
       </c>
@@ -15629,7 +15632,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="497" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="497" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A497">
         <v>496</v>
       </c>
@@ -15667,7 +15670,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="498" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="498" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A498">
         <v>497</v>
       </c>
@@ -15696,7 +15699,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="499" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="499" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A499">
         <v>498</v>
       </c>
@@ -15725,7 +15728,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="500" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="500" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A500">
         <v>499</v>
       </c>
@@ -15754,7 +15757,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="501" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="501" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A501">
         <v>500</v>
       </c>
@@ -15786,7 +15789,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="502" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="502" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A502">
         <v>501</v>
       </c>
@@ -15815,7 +15818,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="503" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="503" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A503">
         <v>502</v>
       </c>
@@ -15853,7 +15856,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="504" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="504" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A504">
         <v>503</v>
       </c>
@@ -15883,7 +15886,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O504" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>